<commit_message>
update output schedule PFP-C
</commit_message>
<xml_diff>
--- a/PFP-C/Input data and Generated Schedule/104.xlsx
+++ b/PFP-C/Input data and Generated Schedule/104.xlsx
@@ -50376,7 +50376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50401,7 +50401,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>objective all vehicle travel individually</t>
+          <t>objective_all_vehicle_travel_individually</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -50411,7 +50411,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>objective LLA</t>
+          <t>objective_LLA</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -50421,11 +50421,131 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>objective lb</t>
+          <t>objective_lb</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>86.27600000000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>max_charge_5</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>mean_charge_5</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>max_charge_10</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>mean_charge_10</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>max_charge_15</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>mean_charge_15</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>max_charge_20</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>mean_charge_20</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>max_charge_25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>mean_charge_25</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>max_charge_30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>mean_charge_30</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -72503,7 +72623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72539,25 +72659,20 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>before_due_time_(minute)</t>
+          <t>duration_trip_alone_(minute)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>duration_trip_alone_(minute)</t>
+          <t>Saving_time_(minute)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Saving_time_(minute)</t>
+          <t>Saving_time(%)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Saving_time(%)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Exit</t>
         </is>
@@ -72590,18 +72705,15 @@
         <v>7.392405063291145</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>344.7484984984985</v>
       </c>
       <c r="I2" t="n">
-        <v>344.7484984984985</v>
+        <v>4.384384384384388</v>
       </c>
       <c r="J2" t="n">
-        <v>4.384384384384388</v>
-      </c>
-      <c r="K2" t="n">
         <v>1.271763155888983</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -72634,18 +72746,15 @@
         <v>7.953020134228177</v>
       </c>
       <c r="H3" t="n">
-        <v>-9.554360850815556</v>
+        <v>253.2297297297297</v>
       </c>
       <c r="I3" t="n">
-        <v>253.2297297297297</v>
+        <v>3.558558558558553</v>
       </c>
       <c r="J3" t="n">
-        <v>3.558558558558553</v>
-      </c>
-      <c r="K3" t="n">
         <v>1.4052688688475</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -72678,18 +72787,15 @@
         <v>9.999999999999989</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>303.3468468468469</v>
       </c>
       <c r="I4" t="n">
-        <v>303.3468468468469</v>
+        <v>5.135135135135129</v>
       </c>
       <c r="J4" t="n">
-        <v>5.135135135135129</v>
-      </c>
-      <c r="K4" t="n">
         <v>1.692826277415617</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -72722,18 +72828,15 @@
         <v>1.328976034858386</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>405.9617117117117</v>
       </c>
       <c r="I5" t="n">
-        <v>405.9617117117117</v>
+        <v>0.9159159159159149</v>
       </c>
       <c r="J5" t="n">
-        <v>0.9159159159159149</v>
-      </c>
-      <c r="K5" t="n">
         <v>0.225616330183951</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -72766,18 +72869,15 @@
         <v>7.036144578313269</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>355.8445945945945</v>
       </c>
       <c r="I6" t="n">
-        <v>355.8445945945945</v>
+        <v>4.384384384384394</v>
       </c>
       <c r="J6" t="n">
-        <v>4.384384384384394</v>
-      </c>
-      <c r="K6" t="n">
         <v>1.232106501260592</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -72810,18 +72910,15 @@
         <v>7.710843373493982</v>
       </c>
       <c r="H7" t="n">
-        <v>-9.986251403484971</v>
+        <v>358.5472972972973</v>
       </c>
       <c r="I7" t="n">
-        <v>358.5472972972973</v>
+        <v>4.804804804804808</v>
       </c>
       <c r="J7" t="n">
-        <v>4.804804804804808</v>
-      </c>
-      <c r="K7" t="n">
         <v>1.340075588638673</v>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -72854,18 +72951,15 @@
         <v>2.510121457489872</v>
       </c>
       <c r="H8" t="n">
-        <v>-7.425248066585823</v>
+        <v>197.1118618618618</v>
       </c>
       <c r="I8" t="n">
-        <v>197.1118618618618</v>
+        <v>0.9309309309309284</v>
       </c>
       <c r="J8" t="n">
-        <v>0.9309309309309284</v>
-      </c>
-      <c r="K8" t="n">
         <v>0.4722855956702064</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>p7</t>
         </is>
@@ -72898,18 +72992,15 @@
         <v>5.459459459459458</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>170.4316816816817</v>
       </c>
       <c r="I9" t="n">
-        <v>170.4316816816817</v>
+        <v>1.516516516516516</v>
       </c>
       <c r="J9" t="n">
-        <v>1.516516516516516</v>
-      </c>
-      <c r="K9" t="n">
         <v>0.8898090434552782</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>p7</t>
         </is>
@@ -72942,18 +73033,15 @@
         <v>7.119999999999996</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>447.072072072072</v>
       </c>
       <c r="I10" t="n">
-        <v>447.072072072072</v>
+        <v>5.345345345345343</v>
       </c>
       <c r="J10" t="n">
-        <v>5.345345345345343</v>
-      </c>
-      <c r="K10" t="n">
         <v>1.195633921074726</v>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -72986,18 +73074,15 @@
         <v>6.531645569620253</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.8750281150698243</v>
+        <v>326.7304804804805</v>
       </c>
       <c r="I11" t="n">
-        <v>326.7304804804805</v>
+        <v>3.873873873873873</v>
       </c>
       <c r="J11" t="n">
-        <v>3.873873873873873</v>
-      </c>
-      <c r="K11" t="n">
         <v>1.185648142829241</v>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -73030,18 +73115,15 @@
         <v>4.594594594594593</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>178.5397897897898</v>
       </c>
       <c r="I12" t="n">
-        <v>178.5397897897898</v>
+        <v>1.276276276276276</v>
       </c>
       <c r="J12" t="n">
-        <v>1.276276276276276</v>
-      </c>
-      <c r="K12" t="n">
         <v>0.7148413682904775</v>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>p7</t>
         </is>
@@ -73074,18 +73156,15 @@
         <v>4.867469879518081</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>355.8445945945947</v>
       </c>
       <c r="I13" t="n">
-        <v>355.8445945945947</v>
+        <v>3.033033033033039</v>
       </c>
       <c r="J13" t="n">
-        <v>3.033033033033039</v>
-      </c>
-      <c r="K13" t="n">
         <v>0.8523476481323261</v>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -73118,18 +73197,15 @@
         <v>7.953020134228177</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>274.2507507507507</v>
       </c>
       <c r="I14" t="n">
-        <v>274.2507507507507</v>
+        <v>3.558558558558553</v>
       </c>
       <c r="J14" t="n">
-        <v>3.558558558558553</v>
-      </c>
-      <c r="K14" t="n">
         <v>1.297556542258185</v>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -73162,18 +73238,15 @@
         <v>8.640350877193004</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>393.051051051051</v>
       </c>
       <c r="I15" t="n">
-        <v>393.051051051051</v>
+        <v>5.915915915915931</v>
       </c>
       <c r="J15" t="n">
-        <v>5.915915915915931</v>
-      </c>
-      <c r="K15" t="n">
         <v>1.5051265987195</v>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -73206,18 +73279,15 @@
         <v>4.576271186440676</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>303.6381381381381</v>
       </c>
       <c r="I16" t="n">
-        <v>303.6381381381381</v>
+        <v>2.432432432432431</v>
       </c>
       <c r="J16" t="n">
-        <v>2.432432432432431</v>
-      </c>
-      <c r="K16" t="n">
         <v>0.8010958199611316</v>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -73250,18 +73320,15 @@
         <v>3.076923076923079</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.9382298504816617</v>
+        <v>258.6343843843844</v>
       </c>
       <c r="I17" t="n">
-        <v>258.6343843843844</v>
+        <v>1.381381381381382</v>
       </c>
       <c r="J17" t="n">
-        <v>1.381381381381382</v>
-      </c>
-      <c r="K17" t="n">
         <v>0.5341058516521001</v>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -73294,18 +73361,15 @@
         <v>6.535087719298266</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>399.057057057057</v>
       </c>
       <c r="I18" t="n">
-        <v>399.057057057057</v>
+        <v>4.474474474474488</v>
       </c>
       <c r="J18" t="n">
-        <v>4.474474474474488</v>
-      </c>
-      <c r="K18" t="n">
         <v>1.121261833451232</v>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -73338,18 +73402,15 @@
         <v>6.900584795321631</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>299.7432432432433</v>
       </c>
       <c r="I19" t="n">
-        <v>299.7432432432433</v>
+        <v>3.54354354354354</v>
       </c>
       <c r="J19" t="n">
-        <v>3.54354354354354</v>
-      </c>
-      <c r="K19" t="n">
         <v>1.182192967955556</v>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -73382,18 +73443,15 @@
         <v>4.865771812080538</v>
       </c>
       <c r="H20" t="n">
-        <v>-9.061750166488196</v>
+        <v>259.8363363363364</v>
       </c>
       <c r="I20" t="n">
-        <v>259.8363363363364</v>
+        <v>2.177177177177177</v>
       </c>
       <c r="J20" t="n">
-        <v>2.177177177177177</v>
-      </c>
-      <c r="K20" t="n">
         <v>0.8379032770686095</v>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -73426,18 +73484,15 @@
         <v>8.607594936708868</v>
       </c>
       <c r="H21" t="n">
-        <v>-6.15545617997617</v>
+        <v>330.9346846846847</v>
       </c>
       <c r="I21" t="n">
-        <v>330.9346846846847</v>
+        <v>5.10510510510511</v>
       </c>
       <c r="J21" t="n">
-        <v>5.10510510510511</v>
-      </c>
-      <c r="K21" t="n">
         <v>1.542632229670718</v>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -73470,18 +73525,15 @@
         <v>7.468354430379756</v>
       </c>
       <c r="H22" t="n">
-        <v>-11.60775235952553</v>
+        <v>339.3430930930931</v>
       </c>
       <c r="I22" t="n">
-        <v>339.3430930930931</v>
+        <v>4.429429429429435</v>
       </c>
       <c r="J22" t="n">
-        <v>4.429429429429435</v>
-      </c>
-      <c r="K22" t="n">
         <v>1.305295295406026</v>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -73514,18 +73566,15 @@
         <v>7.489878542510123</v>
       </c>
       <c r="H23" t="n">
-        <v>-15.85842662603113</v>
+        <v>218.7334834834836</v>
       </c>
       <c r="I23" t="n">
-        <v>218.7334834834836</v>
+        <v>2.777777777777778</v>
       </c>
       <c r="J23" t="n">
-        <v>2.777777777777778</v>
-      </c>
-      <c r="K23" t="n">
         <v>1.269937155272126</v>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>p7</t>
         </is>
@@ -73558,18 +73607,15 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
+        <v>162.0232732732733</v>
+      </c>
+      <c r="I24" t="n">
         <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>162.0232732732733</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>p7</t>
         </is>
@@ -73602,18 +73648,15 @@
         <v>5.156626506024106</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>357.0457957957958</v>
       </c>
       <c r="I25" t="n">
-        <v>357.0457957957958</v>
+        <v>3.213213213213219</v>
       </c>
       <c r="J25" t="n">
-        <v>3.213213213213219</v>
-      </c>
-      <c r="K25" t="n">
         <v>0.899944279150942</v>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -73646,18 +73689,15 @@
         <v>9.180000000000026</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>436.8618618618618</v>
       </c>
       <c r="I26" t="n">
-        <v>436.8618618618618</v>
+        <v>6.891891891891913</v>
       </c>
       <c r="J26" t="n">
-        <v>6.891891891891913</v>
-      </c>
-      <c r="K26" t="n">
         <v>1.577590651314664</v>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -73690,18 +73730,15 @@
         <v>8.67469879518073</v>
       </c>
       <c r="H27" t="n">
-        <v>-2.744207353056709</v>
+        <v>369.9587087087087</v>
       </c>
       <c r="I27" t="n">
-        <v>369.9587087087087</v>
+        <v>5.40540540540541</v>
       </c>
       <c r="J27" t="n">
-        <v>5.40540540540541</v>
-      </c>
-      <c r="K27" t="n">
         <v>1.461083433951927</v>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -73734,18 +73771,15 @@
         <v>8.962025316455708</v>
       </c>
       <c r="H28" t="n">
-        <v>-14.07701410642522</v>
+        <v>339.9436936936937</v>
       </c>
       <c r="I28" t="n">
-        <v>339.9436936936937</v>
+        <v>5.315315315315323</v>
       </c>
       <c r="J28" t="n">
-        <v>5.315315315315323</v>
-      </c>
-      <c r="K28" t="n">
         <v>1.56358697452546</v>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -73778,18 +73812,15 @@
         <v>8.804664723032083</v>
       </c>
       <c r="H29" t="n">
-        <v>-18.54421856513517</v>
+        <v>295.8385885885886</v>
       </c>
       <c r="I29" t="n">
-        <v>295.8385885885886</v>
+        <v>4.534534534534542</v>
       </c>
       <c r="J29" t="n">
-        <v>4.534534534534542</v>
-      </c>
-      <c r="K29" t="n">
         <v>1.532773177484478</v>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>p7</t>
         </is>
@@ -73822,18 +73853,15 @@
         <v>8.506024096385557</v>
       </c>
       <c r="H30" t="n">
-        <v>-6.484480897975686</v>
+        <v>362.7515015015015</v>
       </c>
       <c r="I30" t="n">
-        <v>362.7515015015015</v>
+        <v>5.300300300300309</v>
       </c>
       <c r="J30" t="n">
-        <v>5.300300300300309</v>
-      </c>
-      <c r="K30" t="n">
         <v>1.461138073408738</v>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -73866,18 +73894,15 @@
         <v>8.06100217864924</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>395.1509009009009</v>
       </c>
       <c r="I31" t="n">
-        <v>395.1509009009009</v>
+        <v>5.555555555555556</v>
       </c>
       <c r="J31" t="n">
-        <v>5.555555555555556</v>
-      </c>
-      <c r="K31" t="n">
         <v>1.405932655825786</v>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -73910,18 +73935,15 @@
         <v>10.00000000000002</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>438.0630630630631</v>
       </c>
       <c r="I32" t="n">
-        <v>438.0630630630631</v>
+        <v>7.50750750750752</v>
       </c>
       <c r="J32" t="n">
-        <v>7.50750750750752</v>
-      </c>
-      <c r="K32" t="n">
         <v>1.713796058269069</v>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -73954,18 +73976,15 @@
         <v>5.482456140350877</v>
       </c>
       <c r="H33" t="n">
-        <v>-19.14441574543253</v>
+        <v>402.3603603603603</v>
       </c>
       <c r="I33" t="n">
-        <v>402.3603603603603</v>
+        <v>3.753753753753753</v>
       </c>
       <c r="J33" t="n">
-        <v>3.753753753753753</v>
-      </c>
-      <c r="K33" t="n">
         <v>0.9329332915379218</v>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -73998,18 +74017,15 @@
         <v>10.00000000000002</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>434.1591591591592</v>
       </c>
       <c r="I34" t="n">
-        <v>434.1591591591592</v>
+        <v>7.50750750750752</v>
       </c>
       <c r="J34" t="n">
-        <v>7.50750750750752</v>
-      </c>
-      <c r="K34" t="n">
         <v>1.729206294310914</v>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -74042,18 +74058,15 @@
         <v>6.688741721854304</v>
       </c>
       <c r="H35" t="n">
-        <v>-26.86447908187483</v>
+        <v>266.43993993994</v>
       </c>
       <c r="I35" t="n">
-        <v>266.43993993994</v>
+        <v>3.033033033033032</v>
       </c>
       <c r="J35" t="n">
-        <v>3.033033033033032</v>
-      </c>
-      <c r="K35" t="n">
         <v>1.138355245732576</v>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>p7</t>
         </is>
@@ -74086,18 +74099,15 @@
         <v>4.771084337349406</v>
       </c>
       <c r="H36" t="n">
-        <v>-1.519269286660574</v>
+        <v>361.2499999999999</v>
       </c>
       <c r="I36" t="n">
-        <v>361.2499999999999</v>
+        <v>2.972972972972979</v>
       </c>
       <c r="J36" t="n">
-        <v>2.972972972972979</v>
-      </c>
-      <c r="K36" t="n">
         <v>0.8229682970167416</v>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -74130,18 +74140,15 @@
         <v>7.900000000000008</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>423.948948948949</v>
       </c>
       <c r="I37" t="n">
-        <v>423.948948948949</v>
+        <v>5.930930930930938</v>
       </c>
       <c r="J37" t="n">
-        <v>5.930930930930938</v>
-      </c>
-      <c r="K37" t="n">
         <v>1.398972905967772</v>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -74174,18 +74181,15 @@
         <v>9.999999999999986</v>
       </c>
       <c r="H38" t="n">
-        <v>-9.192699264706221</v>
+        <v>288.0645645645646</v>
       </c>
       <c r="I38" t="n">
-        <v>288.0645645645646</v>
+        <v>4.474474474474468</v>
       </c>
       <c r="J38" t="n">
-        <v>4.474474474474468</v>
-      </c>
-      <c r="K38" t="n">
         <v>1.553288750123792</v>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -74218,18 +74222,15 @@
         <v>2.07357859531772</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>249.0247747747748</v>
       </c>
       <c r="I39" t="n">
-        <v>249.0247747747748</v>
+        <v>0.9309309309309284</v>
       </c>
       <c r="J39" t="n">
-        <v>0.9309309309309284</v>
-      </c>
-      <c r="K39" t="n">
         <v>0.3738306486866174</v>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -74262,18 +74263,15 @@
         <v>9.999999999999996</v>
       </c>
       <c r="H40" t="n">
-        <v>-20.16073450149611</v>
+        <v>254.4301801801802</v>
       </c>
       <c r="I40" t="n">
-        <v>254.4301801801802</v>
+        <v>4.489489489489488</v>
       </c>
       <c r="J40" t="n">
-        <v>4.489489489489488</v>
-      </c>
-      <c r="K40" t="n">
         <v>1.764527103785471</v>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -74306,18 +74304,15 @@
         <v>10.00000000000001</v>
       </c>
       <c r="H41" t="n">
-        <v>-6.945511046845468</v>
+        <v>412.8708708708709</v>
       </c>
       <c r="I41" t="n">
-        <v>412.8708708708709</v>
+        <v>6.846846846846852</v>
       </c>
       <c r="J41" t="n">
-        <v>6.846846846846852</v>
-      </c>
-      <c r="K41" t="n">
         <v>1.658350668431696</v>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -74350,18 +74345,15 @@
         <v>1.315789473684209</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>297.3408408408409</v>
       </c>
       <c r="I42" t="n">
-        <v>297.3408408408409</v>
+        <v>0.6756756756756745</v>
       </c>
       <c r="J42" t="n">
-        <v>0.6756756756756745</v>
-      </c>
-      <c r="K42" t="n">
         <v>0.227239444727792</v>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -74394,18 +74386,15 @@
         <v>5.40540540540541</v>
       </c>
       <c r="H43" t="n">
-        <v>-12.07518793597444</v>
+        <v>146.4076576576576</v>
       </c>
       <c r="I43" t="n">
-        <v>146.4076576576576</v>
+        <v>1.501501501501503</v>
       </c>
       <c r="J43" t="n">
-        <v>1.501501501501503</v>
-      </c>
-      <c r="K43" t="n">
         <v>1.025562136245931</v>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>p7</t>
         </is>
@@ -74438,18 +74427,15 @@
         <v>4.940000000000015</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>445.2702702702703</v>
       </c>
       <c r="I44" t="n">
-        <v>445.2702702702703</v>
+        <v>3.70870870870872</v>
       </c>
       <c r="J44" t="n">
-        <v>3.70870870870872</v>
-      </c>
-      <c r="K44" t="n">
         <v>0.8329118192547657</v>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -74482,18 +74468,15 @@
         <v>4.727668845315915</v>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>399.3551051051051</v>
       </c>
       <c r="I45" t="n">
-        <v>399.3551051051051</v>
+        <v>3.258258258258266</v>
       </c>
       <c r="J45" t="n">
-        <v>3.258258258258266</v>
-      </c>
-      <c r="K45" t="n">
         <v>0.8158799566117314</v>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -74526,18 +74509,15 @@
         <v>7.376237623762377</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>361.5585585585586</v>
       </c>
       <c r="I46" t="n">
-        <v>361.5585585585586</v>
+        <v>4.474474474474475</v>
       </c>
       <c r="J46" t="n">
-        <v>4.474474474474475</v>
-      </c>
-      <c r="K46" t="n">
         <v>1.237551806908695</v>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -74570,18 +74550,15 @@
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>-8.670939573111127</v>
+        <v>295.2252252252252</v>
       </c>
       <c r="I47" t="n">
-        <v>295.2252252252252</v>
+        <v>0</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
       </c>
-      <c r="K47" t="n">
-        <v>0</v>
-      </c>
-      <c r="L47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -74614,18 +74591,15 @@
         <v>8.713450292397649</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>303.6471471471472</v>
       </c>
       <c r="I48" t="n">
-        <v>303.6471471471472</v>
+        <v>4.474474474474468</v>
       </c>
       <c r="J48" t="n">
-        <v>4.474474474474468</v>
-      </c>
-      <c r="K48" t="n">
         <v>1.47357698450766</v>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>p10</t>
         </is>
@@ -74658,18 +74632,15 @@
         <v>6.168674698795186</v>
       </c>
       <c r="H49" t="n">
-        <v>-26.63623630736834</v>
+        <v>367.256006006006</v>
       </c>
       <c r="I49" t="n">
-        <v>367.256006006006</v>
+        <v>3.843843843843847</v>
       </c>
       <c r="J49" t="n">
-        <v>3.843843843843847</v>
-      </c>
-      <c r="K49" t="n">
         <v>1.04663879718307</v>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -74702,18 +74673,15 @@
         <v>6.912751677852349</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>259.5360360360361</v>
       </c>
       <c r="I50" t="n">
-        <v>259.5360360360361</v>
+        <v>3.093093093093092</v>
       </c>
       <c r="J50" t="n">
-        <v>3.093093093093092</v>
-      </c>
-      <c r="K50" t="n">
         <v>1.191777889627482</v>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>p9</t>
         </is>
@@ -74746,18 +74714,15 @@
         <v>6.187290969899667</v>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>255.0307807807808</v>
       </c>
       <c r="I51" t="n">
-        <v>255.0307807807808</v>
+        <v>2.777777777777778</v>
       </c>
       <c r="J51" t="n">
-        <v>2.777777777777778</v>
-      </c>
-      <c r="K51" t="n">
         <v>1.089193143381974</v>
       </c>
-      <c r="L51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>p8</t>
         </is>
@@ -74774,7 +74739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74800,20 +74765,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>before_due_time_(minute)</t>
+          <t>duration_trip_alone_(minute)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>duration_trip_alone_(minute)</t>
+          <t>Saving_time_(minute)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Saving_time_(minute)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Saving_time(%)</t>
         </is>
@@ -74846,9 +74806,6 @@
       <c r="H2" t="n">
         <v>50</v>
       </c>
-      <c r="I2" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -74869,15 +74826,12 @@
         <v>6.492533781073276</v>
       </c>
       <c r="F3" t="n">
-        <v>-4.890437945690426</v>
+        <v>323.1089039039039</v>
       </c>
       <c r="G3" t="n">
-        <v>323.1089039039039</v>
+        <v>3.728528528528531</v>
       </c>
       <c r="H3" t="n">
-        <v>3.728528528528531</v>
-      </c>
-      <c r="I3" t="n">
         <v>1.116078810021528</v>
       </c>
     </row>
@@ -74900,15 +74854,12 @@
         <v>2.6389588277631</v>
       </c>
       <c r="F4" t="n">
-        <v>7.436861848447185</v>
+        <v>79.13864982774064</v>
       </c>
       <c r="G4" t="n">
-        <v>79.13864982774064</v>
+        <v>1.873723992729907</v>
       </c>
       <c r="H4" t="n">
-        <v>1.873723992729907</v>
-      </c>
-      <c r="I4" t="n">
         <v>0.4496937179302971</v>
       </c>
     </row>
@@ -74931,17 +74882,14 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>-26.86447908187483</v>
+        <v>146.4076576576576</v>
       </c>
       <c r="G5" t="n">
-        <v>146.4076576576576</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -74962,15 +74910,12 @@
         <v>4.885602409638564</v>
       </c>
       <c r="F6" t="n">
-        <v>-8.964047518143929</v>
+        <v>261.4872372372373</v>
       </c>
       <c r="G6" t="n">
-        <v>261.4872372372373</v>
+        <v>2.777777777777778</v>
       </c>
       <c r="H6" t="n">
-        <v>2.777777777777778</v>
-      </c>
-      <c r="I6" t="n">
         <v>0.8415143698345386</v>
       </c>
     </row>
@@ -74993,15 +74938,12 @@
         <v>6.974448128082809</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>335.1388888888889</v>
       </c>
       <c r="G7" t="n">
-        <v>335.1388888888889</v>
+        <v>3.7987987987988</v>
       </c>
       <c r="H7" t="n">
-        <v>3.7987987987988</v>
-      </c>
-      <c r="I7" t="n">
         <v>1.193705905351104</v>
       </c>
     </row>
@@ -75024,15 +74966,12 @@
         <v>8.58220222662804</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>387.2779654654655</v>
       </c>
       <c r="G8" t="n">
-        <v>387.2779654654655</v>
+        <v>5.030030030030034</v>
       </c>
       <c r="H8" t="n">
-        <v>5.030030030030034</v>
-      </c>
-      <c r="I8" t="n">
         <v>1.461124413544536</v>
       </c>
     </row>
@@ -75055,15 +74994,12 @@
         <v>10.00000000000002</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>447.072072072072</v>
       </c>
       <c r="G9" t="n">
-        <v>447.072072072072</v>
+        <v>7.50750750750752</v>
       </c>
       <c r="H9" t="n">
-        <v>7.50750750750752</v>
-      </c>
-      <c r="I9" t="n">
         <v>1.764527103785471</v>
       </c>
     </row>

</xml_diff>